<commit_message>
Livrable final — README, script de tests, dépendances
- README.md : index du dépôt, commandes de chaque livrable, liste
  exhaustive des {{VARIABLES}}, actions restant humaines, scores des
  validations et des tests
- tests.sh : lance vérifications juridiques, Google Ads, fiche de poste,
  129 tests Python (couverture classificateur ≥ 85 %) et contrôle des
  placeholders
- requirements.txt complété (docxtpl, reportlab), .gitignore (sorties,
  .base_id)

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNriugc5W7v9SCzgqVT7Aq
</commit_message>
<xml_diff>
--- a/juridique/registre-traitements-rgpd.xlsx
+++ b/juridique/registre-traitements-rgpd.xlsx
@@ -555,7 +555,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -800,12 +800,12 @@
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -900,12 +900,12 @@
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -1000,12 +1000,12 @@
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -1100,12 +1100,12 @@
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -1200,12 +1200,12 @@
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Site public complet prêt pour Cloudflare Pages
- site/build.py : construit dist/ (accueil, CGV, confidentialité, mandat,
  mentions légales, 404, robots, sitemap, en-têtes de sécurité, image de partage)
  depuis les sources juridiques Markdown ; refuse de publier si une valeur
  obligatoire manque ; mode --apercu pour prévisualiser
- site/config.json : valeurs publiées (identité de la société, sous-traitants)
- juridique/variables.py : variables et blocs conditionnels partagés entre
  documents Word et site (téléphone, TVA, assurance, médiateur, ligne 2FA
  facultatifs, formulations adaptées)
- Formulaire : envoi par la messagerie du visiteur tant que Formspree n'est
  pas configuré
- Politique de confidentialité et registre : hébergeur du site ajouté
- 27 tests, vnu et html-validate sans erreur, Lighthouse 97-100

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y1ccwmnSo11YFZ7zwBaNdA
</commit_message>
<xml_diff>
--- a/juridique/registre-traitements-rgpd.xlsx
+++ b/juridique/registre-traitements-rgpd.xlsx
@@ -555,7 +555,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -800,12 +800,12 @@
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -900,12 +900,12 @@
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -1000,12 +1000,12 @@
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -1100,12 +1100,12 @@
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -1165,7 +1165,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Formspree (réception du formulaire) ; service de messagerie ; outil de visioconférence.</t>
+          <t>Hébergeur du site ; Formspree (réception du formulaire, si activé) ; service de messagerie ; outil de visioconférence.</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -1200,12 +1200,12 @@
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1422,25 +1422,52 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>Hébergeur du site</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Hébergement et diffusion du site internet</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>{{HEBERGEUR_NOM}}</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>{{HEBERGEUR_LOCALISATION}}</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Conditions du fournisseur (art. 28) ; clauses contractuelles types ; aucune donnée de dossier</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>Formspree</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Formulaire de contact</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>{{FORMSPREE_ENTITE}}</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>{{FORMSPREE_HEBERGEMENT}}</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>Clauses contractuelles types (États-Unis)</t>
         </is>

</xml_diff>

<commit_message>
Juridique : analyse d'impact RGPD, dossier de consultation de l'avocat ; procédure 13 d'accueil du parent
- juridique/aipd-relais.md et .docx : AIPD selon la méthode CNIL (critères,
  flux, bases légales, durées, risques, mesures avant le premier client).
- juridique/consultation-avocat.md et .docx : contexte, pièces et huit
  questions (accès bancaires et DSP2, identifiants et FranceConnect, HDS,
  signature électronique, paiement avant mandat, activités réglementées,
  transfert du contrat, loi applicable).
- procedures/13-accueil-parent-et-mandat.md : appel à trois, mot de code
  contre les faux appels, envoi du mandat prérempli, relances, remboursement
  à J+30 ; index mis à jour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013iLDprCHrWFcERNnonBWVW
</commit_message>
<xml_diff>
--- a/juridique/registre-traitements-rgpd.xlsx
+++ b/juridique/registre-traitements-rgpd.xlsx
@@ -555,7 +555,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
     </row>
@@ -800,12 +800,12 @@
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
     </row>
@@ -900,12 +900,12 @@
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
     </row>
@@ -1000,12 +1000,12 @@
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
     </row>
@@ -1100,12 +1100,12 @@
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
     </row>
@@ -1200,12 +1200,12 @@
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
     </row>

</xml_diff>